<commit_message>
chore(live-exams): refresh workbook (85 rows)
</commit_message>
<xml_diff>
--- a/live-exam-notifications/Live_Exam_Notifications.xlsx
+++ b/live-exam-notifications/Live_Exam_Notifications.xlsx
@@ -163,7 +163,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -227,6 +227,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -633,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="B2:D20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="12" min="1" max="1"/>
@@ -642,7 +645,6 @@
     <col width="12" customWidth="1" style="12" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="15" customHeight="1" s="13">
       <c r="B2" s="14" t="inlineStr">
         <is>
@@ -653,11 +655,10 @@
     <row r="3" ht="15" customHeight="1" s="13">
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>Currently open and recently closed recruitment and entrance-exam notifications, verified against official portals. Last verified 25 October 2026; refreshed automatically twice a week.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
+          <t>Currently open and recently closed recruitment and entrance-exam notifications, verified against official portals. Last verified 26 October 2026; refreshed automatically twice a week.</t>
+        </is>
+      </c>
+    </row>
     <row r="5" ht="15" customHeight="1" s="13">
       <c r="B5" s="16" t="inlineStr">
         <is>
@@ -684,7 +685,7 @@
     <row r="10" ht="15" customHeight="1" s="13">
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>Status reflects the position on 25 October 2026: green = open, blue = upcoming, grey = dates to be announced, red = recently closed.</t>
+          <t>Status reflects the position on 26 October 2026: green = open, blue = upcoming, grey = dates to be announced, red = recently closed.</t>
         </is>
       </c>
     </row>
@@ -697,7 +698,6 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="13"/>
-    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="13">
       <c r="B15" s="16" t="inlineStr">
         <is>
@@ -785,7 +785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q75"/>
+  <dimension ref="A1:Q86"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="12" min="1" max="1"/>
@@ -7072,263 +7072,1158 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
+      <c r="A73" s="12" t="inlineStr">
         <is>
           <t>Central Govt</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B73" s="12" t="inlineStr">
         <is>
           <t>National Insurance Company Limited (NICL) - conducted through IBPS</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C73" s="12" t="inlineStr">
         <is>
           <t>Recruitment of 321 Administrative Officers (Generalists &amp; Specialists) (Scale I), 2026-27</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D73" s="12" t="inlineStr">
         <is>
           <t>recruitment</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
+      <c r="E73" s="12" t="inlineStr">
         <is>
           <t>321 vacancies (Generalist Officers 200; specialists 121 - Finance 20, Legal 20, IT 21, Automobile 10, Risk 28, Company Secretary 2, Agriculture 20)</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F73" s="12" t="inlineStr">
         <is>
           <t>Graduation/PG with 60% (55% for SC/ST/PwBD); post-wise (CA/CMA, LL.B., B.E./B.Tech./MCA, Agriculture etc.)</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
+      <c r="G73" s="12" t="inlineStr">
         <is>
           <t>21 to 30 years as on 01/10/2026 (born not earlier than 02/10/1996 and not later than 01/10/2005)</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr">
+      <c r="H73" s="12" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
+      <c r="I73" s="12" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr">
+      <c r="J73" s="12" t="inlineStr">
         <is>
           <t>As per Government rules (SC/ST/OBC/PwBD/EWS/ExSM)</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr">
+      <c r="K73" s="12" t="inlineStr">
         <is>
           <t>08/10/2026 to 28/10/2026</t>
         </is>
       </c>
-      <c r="L73" t="inlineStr">
+      <c r="L73" s="12" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="M73" t="inlineStr">
+      <c r="M73" s="12" t="inlineStr">
         <is>
           <t>Phase-I 17/11/2026; Phase-II 22/12/2026</t>
         </is>
       </c>
-      <c r="N73" t="inlineStr">
+      <c r="N73" s="12" t="inlineStr">
         <is>
           <t>https://ibpsreg.ibps.in/niiclsep26/</t>
         </is>
       </c>
-      <c r="O73" t="inlineStr">
+      <c r="O73" s="12" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="P73" t="inlineStr">
+      <c r="P73" s="12" t="inlineStr">
         <is>
           <t>2026-10-25</t>
         </is>
       </c>
-      <c r="Q73" t="inlineStr">
+      <c r="Q73" s="12" t="inlineStr">
         <is>
           <t>Fee Rs.1,000 (Rs.250 for SC/ST/PwBD); basic pay Rs.82,485 per month. Notification dated 07/10/2026; registration through the IBPS portal (organisation code NICL). Prelims + Mains + Interview.</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" s="12" t="inlineStr">
         <is>
           <t>Central Govt</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B74" s="12" t="inlineStr">
         <is>
           <t>Indo-Tibetan Border Police Force (ITBP), Ministry of Home Affairs</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C74" s="12" t="inlineStr">
         <is>
           <t>Recruitment of Meritorious Sportspersons to the post of Constable (General Duty) under Sports Quota-2025 (detailed advertisement dated 03/10/2026)</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D74" s="12" t="inlineStr">
         <is>
           <t>recruitment</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
+      <c r="E74" s="12" t="inlineStr">
         <is>
           <t>126 posts (72 male, 54 female) across 28 sports disciplines</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="F74" s="12" t="inlineStr">
         <is>
           <t>Matriculation (10th pass) or equivalent, plus prescribed sports achievement between 01/01/2024 and 01/11/2026</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr">
+      <c r="G74" s="12" t="inlineStr">
         <is>
           <t>18 to 23 years as on 01/11/2026</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr">
+      <c r="H74" s="12" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr">
+      <c r="I74" s="12" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr">
+      <c r="J74" s="12" t="inlineStr">
         <is>
           <t>5 years (UR/EWS/OBC sportspersons), 8 years (OBC-NCL), 10 years (SC/ST); not open to PwBD or ex-servicemen</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr">
+      <c r="K74" s="12" t="inlineStr">
         <is>
           <t>03/10/2026 to 01/11/2026 (11:59 PM)</t>
         </is>
       </c>
-      <c r="L74" t="inlineStr">
+      <c r="L74" s="12" t="inlineStr">
         <is>
           <t>2026-11-01</t>
         </is>
       </c>
-      <c r="M74" t="inlineStr">
+      <c r="M74" s="12" t="inlineStr">
         <is>
           <t>Sports trials/documentation as per admit card</t>
         </is>
       </c>
-      <c r="N74" t="inlineStr">
+      <c r="N74" s="12" t="inlineStr">
         <is>
           <t>https://recruitment.itbpolice.nic.in</t>
         </is>
       </c>
-      <c r="O74" t="inlineStr">
+      <c r="O74" s="12" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="P74" t="inlineStr">
+      <c r="P74" s="12" t="inlineStr">
         <is>
           <t>2026-10-25</t>
         </is>
       </c>
-      <c r="Q74" t="inlineStr">
+      <c r="Q74" s="12" t="inlineStr">
         <is>
           <t>Pay Level-3 (Rs.21,700-69,100); fee Rs.100 (male UR/OBC/EWS), exempt for women/SC/ST. Online only at recruitment.itbpolice.nic.in.</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="12" t="inlineStr">
         <is>
           <t>Central Govt</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="12" t="inlineStr">
         <is>
           <t>NTA (for Rashtriya Military Schools, Ministry of Defence)</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="12" t="inlineStr">
         <is>
           <t>Rashtriya Military School Common Entrance Test (RMS CET) 2026 - admission to Class VI and IX (2027-28 session)</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D75" s="12" t="inlineStr">
         <is>
           <t>entrance-exam</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="E75" s="12" t="inlineStr">
         <is>
           <t>Admission to Class VI and Class IX in the five Rashtriya Military Schools (Chail, Ajmer, Dholpur, Belgaum, Bengaluru)</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F75" s="12" t="inlineStr">
         <is>
           <t>Class VI: passed/studying Class V; Class IX: passed Class VIII from a recognised school before admission</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
+      <c r="G75" s="12" t="inlineStr">
         <is>
           <t>Class VI: 10 to 13 years as on 31 March of the year of admission; Class IX: 13 to 16 years</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr">
+      <c r="H75" s="12" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr">
+      <c r="I75" s="12" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr">
+      <c r="J75" s="12" t="inlineStr">
         <is>
           <t>Six months relaxation in upper age limit for wards of personnel killed in action</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr">
+      <c r="K75" s="12" t="inlineStr">
         <is>
           <t>23/09/2026 to 20/10/2026 (regular); late-fee window to 25/10/2026 (up to 5:00 PM)</t>
         </is>
       </c>
-      <c r="L75" t="inlineStr">
+      <c r="L75" s="12" t="inlineStr">
         <is>
           <t>2026-10-25</t>
         </is>
       </c>
-      <c r="M75" t="inlineStr">
+      <c r="M75" s="12" t="inlineStr">
         <is>
           <t>13/12/2026</t>
         </is>
       </c>
-      <c r="N75" t="inlineStr">
+      <c r="N75" s="12" t="inlineStr">
         <is>
           <t>https://exams.nta.nic.in/rmscet/</t>
         </is>
       </c>
-      <c r="O75" t="inlineStr">
+      <c r="O75" s="12" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="P75" t="inlineStr">
+      <c r="P75" s="12" t="inlineStr">
         <is>
           <t>2026-10-25</t>
         </is>
       </c>
-      <c r="Q75" t="inlineStr">
+      <c r="Q75" s="12" t="inlineStr">
         <is>
           <t>Regular window closed 20/10/2026; late submission with Rs.500 late fee open to 25/10/2026. Correction 27-28/10/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="B76" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh Public Service Commission (APPSC)</t>
+        </is>
+      </c>
+      <c r="C76" s="22" t="inlineStr">
+        <is>
+          <t>Notification No. 10/2026 - Assistant Director, A.P. Tribal Welfare State Service (General Recruitment)</t>
+        </is>
+      </c>
+      <c r="D76" s="22" t="inlineStr">
+        <is>
+          <t>recruitment</t>
+        </is>
+      </c>
+      <c r="E76" s="22" t="inlineStr">
+        <is>
+          <t>1 provisional vacancy - Assistant Director in A.P. Tribal Welfare State Service (pay Rs 48,440 - 1,37,220)</t>
+        </is>
+      </c>
+      <c r="F76" s="22" t="inlineStr">
+        <is>
+          <t>1st or 2nd class Master's Degree in Social Anthropology / Sociology / Social Work from a recognised university, with at least two publications in national-level academic journals</t>
+        </is>
+      </c>
+      <c r="G76" s="22" t="inlineStr">
+        <is>
+          <t>Not stated in the brief notification - the age clause is in the Detailed Notification (due on or before 13/10/2026); left blank rather than guessed</t>
+        </is>
+      </c>
+      <c r="H76" s="22" t="inlineStr"/>
+      <c r="I76" s="22" t="inlineStr"/>
+      <c r="J76" s="22" t="inlineStr">
+        <is>
+          <t>SC/ST/BC/EWS 5 years; PwBD 10 years; ex-servicemen and regular AP Government employees as per A.P. State and Subordinate Service Rules (relaxation details in the Detailed Notification)</t>
+        </is>
+      </c>
+      <c r="K76" s="22" t="inlineStr">
+        <is>
+          <t>13/10/2026 to 02/11/2026 (11:59 PM)</t>
+        </is>
+      </c>
+      <c r="L76" s="22" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="M76" s="22" t="inlineStr">
+        <is>
+          <t>tba (single-level CBRT, no screening test)</t>
+        </is>
+      </c>
+      <c r="N76" s="22" t="inlineStr">
+        <is>
+          <t>https://psc.ap.gov.in</t>
+        </is>
+      </c>
+      <c r="O76" s="22" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P76" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="Q76" s="22" t="inlineStr">
+        <is>
+          <t>Brief notification dated 15/09/2026; single-level online CBRT only; detailed notification (vacancy break-up, age, community) was due on or before 13/10/2026 and is the crucial date for eligibility</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="B77" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh Public Service Commission (APPSC)</t>
+        </is>
+      </c>
+      <c r="C77" s="22" t="inlineStr">
+        <is>
+          <t>Notification No. 11/2026 - Assistant Director (Forensic Engineering / Physics / Chemistry / Biology), A.P. State Forensic Science Laboratory Service (General Recruitment)</t>
+        </is>
+      </c>
+      <c r="D77" s="22" t="inlineStr">
+        <is>
+          <t>recruitment</t>
+        </is>
+      </c>
+      <c r="E77" s="22" t="inlineStr">
+        <is>
+          <t>8 posts (Forensic Engineering 1 carried forward; Physics 2; Chemistry 2; Biology 3) - pay Rs 57,100 - 1,47,760</t>
+        </is>
+      </c>
+      <c r="F77" s="22" t="inlineStr">
+        <is>
+          <t>Forensic Engineering: B.E/B.Tech in Mechanical, Civil, Structural or Production Engineering; Physics: M.Sc (1st/2nd class) in Physics, Applied Physics, Material Science, Nuclear Physics, Electronics, Instrumentation, Nano Science/Technology or Geo Physics; Chemistry: M.Sc Chemistry or B.Sc with A.I.C. by examination in Forensic Sciences; Biology: M.Sc (1st/2nd class) in Botany/Zoology/Microbiology/Biochemistry/Genetics/Forensic Science. Exceptionally good eyesight (colour blindness a disqualification) and at least five years practical experience in a Forensic Science, Chemistry, Analytical or Police laboratory</t>
+        </is>
+      </c>
+      <c r="G77" s="22" t="inlineStr">
+        <is>
+          <t>Not stated in the brief notification - the age clause is in the Detailed Notification (due on or before 06/10/2026); left blank rather than guessed</t>
+        </is>
+      </c>
+      <c r="H77" s="22" t="inlineStr"/>
+      <c r="I77" s="22" t="inlineStr"/>
+      <c r="J77" s="22" t="inlineStr">
+        <is>
+          <t>SC/ST/BC/EWS 5 years; PwBD 10 years; ex-servicemen and regular AP Government employees as per A.P. State and Subordinate Service Rules (relaxation details in the Detailed Notification)</t>
+        </is>
+      </c>
+      <c r="K77" s="22" t="inlineStr">
+        <is>
+          <t>06/10/2026 to 27/10/2026 (11:59 PM)</t>
+        </is>
+      </c>
+      <c r="L77" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="M77" s="22" t="inlineStr">
+        <is>
+          <t>tba (single-level CBRT, no screening test)</t>
+        </is>
+      </c>
+      <c r="N77" s="22" t="inlineStr">
+        <is>
+          <t>https://psc.ap.gov.in</t>
+        </is>
+      </c>
+      <c r="O77" s="22" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P77" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="Q77" s="22" t="inlineStr">
+        <is>
+          <t>Brief notification dated 15/09/2026; applications close 27/10/2026; detailed notification (vacancy break-up, age, community) was due on or before 06/10/2026 and is the crucial date for eligibility</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="B78" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh Public Service Commission (APPSC)</t>
+        </is>
+      </c>
+      <c r="C78" s="22" t="inlineStr">
+        <is>
+          <t>Notification No. 29/2026 - Deputy Commissioner of Endowments and Assistant Commissioner of Endowments, A.P. Charitable and Hindu Religious Institutions and Endowments Service</t>
+        </is>
+      </c>
+      <c r="D78" s="22" t="inlineStr">
+        <is>
+          <t>recruitment</t>
+        </is>
+      </c>
+      <c r="E78" s="22" t="inlineStr">
+        <is>
+          <t>11 posts (Deputy Commissioner of Endowments 6 - Rs 65,360-1,54,980; Assistant Commissioner of Endowments 5 - Rs 48,440-1,37,220)</t>
+        </is>
+      </c>
+      <c r="F78" s="22" t="inlineStr">
+        <is>
+          <t>Practising advocate - Deputy Commissioner: at least 5 years' practice in the High Court of A.P. or the Supreme Court; Assistant Commissioner: advocate of the A.P. High Court for at least 3 years. Candidates must profess the Hindu religion (s.29(3), AP Charitable and Hindu Religious Institutions and Endowments Act, 1987)</t>
+        </is>
+      </c>
+      <c r="G78" s="22" t="inlineStr">
+        <is>
+          <t>28-44 years (Age as on 01/07/2026)</t>
+        </is>
+      </c>
+      <c r="H78" s="22" t="n">
+        <v>28</v>
+      </c>
+      <c r="I78" s="22" t="n">
+        <v>44</v>
+      </c>
+      <c r="J78" s="22" t="inlineStr">
+        <is>
+          <t>SC/ST/BC/EWS 5 years; PwBD 10 years; ex-servicemen and regular AP Government employees as per A.P. State and Subordinate Service Rules (relaxation details in the Detailed Notification)</t>
+        </is>
+      </c>
+      <c r="K78" s="22" t="inlineStr">
+        <is>
+          <t>02/11/2026 to 22/11/2026 (11:59 PM)</t>
+        </is>
+      </c>
+      <c r="L78" s="22" t="inlineStr">
+        <is>
+          <t>2026-11-22</t>
+        </is>
+      </c>
+      <c r="M78" s="22" t="inlineStr">
+        <is>
+          <t>tba (single-level CBRT, no screening test)</t>
+        </is>
+      </c>
+      <c r="N78" s="22" t="inlineStr">
+        <is>
+          <t>https://psc.ap.gov.in</t>
+        </is>
+      </c>
+      <c r="O78" s="22" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="P78" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="Q78" s="22" t="inlineStr">
+        <is>
+          <t>Brief notification dated 13/10/2026; applications open 02/11/2026; BC-C and BC-E candidates are not eligible to the Endowments posts under the department special rules; detailed notification due on or before 02/11/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="B79" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh Public Service Commission (APPSC)</t>
+        </is>
+      </c>
+      <c r="C79" s="22" t="inlineStr">
+        <is>
+          <t>Notification No. 31/2026 - Assistant Director (Mines), A.P. Mines and Geology Service</t>
+        </is>
+      </c>
+      <c r="D79" s="22" t="inlineStr">
+        <is>
+          <t>recruitment</t>
+        </is>
+      </c>
+      <c r="E79" s="22" t="inlineStr">
+        <is>
+          <t>1 provisional vacancy - Assistant Director (Mines), pay Rs 57,100 - 1,47,760</t>
+        </is>
+      </c>
+      <c r="F79" s="22" t="inlineStr">
+        <is>
+          <t>Degree in Mining Engineering from a recognised university, or Diploma in Mining Engineering from Indian School of Mines, Dhanbad or equivalent</t>
+        </is>
+      </c>
+      <c r="G79" s="22" t="inlineStr">
+        <is>
+          <t>18-44 years (Age as on 01/07/2026)</t>
+        </is>
+      </c>
+      <c r="H79" s="22" t="n">
+        <v>18</v>
+      </c>
+      <c r="I79" s="22" t="n">
+        <v>44</v>
+      </c>
+      <c r="J79" s="22" t="inlineStr">
+        <is>
+          <t>SC/ST/BC/EWS 5 years; PwBD 10 years; ex-servicemen and regular AP Government employees as per A.P. State and Subordinate Service Rules (relaxation details in the Detailed Notification)</t>
+        </is>
+      </c>
+      <c r="K79" s="22" t="inlineStr">
+        <is>
+          <t>06/11/2026 to 26/11/2026 (11:59 PM)</t>
+        </is>
+      </c>
+      <c r="L79" s="22" t="inlineStr">
+        <is>
+          <t>2026-11-26</t>
+        </is>
+      </c>
+      <c r="M79" s="22" t="inlineStr">
+        <is>
+          <t>tba (single-level CBRT, no screening test)</t>
+        </is>
+      </c>
+      <c r="N79" s="22" t="inlineStr">
+        <is>
+          <t>https://psc.ap.gov.in</t>
+        </is>
+      </c>
+      <c r="O79" s="22" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="P79" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="Q79" s="22" t="inlineStr">
+        <is>
+          <t>Brief notification dated 13/10/2026; applications open 06/11/2026; detailed notification due on or before 06/11/2026 and is the crucial date for eligibility</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="B80" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh Public Service Commission (APPSC)</t>
+        </is>
+      </c>
+      <c r="C80" s="22" t="inlineStr">
+        <is>
+          <t>Notification No. 32/2026 - Technical Assistant, A.P. Mines and Geology Sub-Service</t>
+        </is>
+      </c>
+      <c r="D80" s="22" t="inlineStr">
+        <is>
+          <t>recruitment</t>
+        </is>
+      </c>
+      <c r="E80" s="22" t="inlineStr">
+        <is>
+          <t>36 provisional vacancies - Technical Assistant in A.P. Mines and Geology Sub-Service, pay Rs 35,570 - 1,09,910</t>
+        </is>
+      </c>
+      <c r="F80" s="22" t="inlineStr">
+        <is>
+          <t>B.Sc degree in Geology from a recognised university; practical experience of not less than one year in investigation of mineral deposits, geological mapping, mining or underground water resources preferred</t>
+        </is>
+      </c>
+      <c r="G80" s="22" t="inlineStr">
+        <is>
+          <t>18-44 years (Age as on 01/07/2026)</t>
+        </is>
+      </c>
+      <c r="H80" s="22" t="n">
+        <v>18</v>
+      </c>
+      <c r="I80" s="22" t="n">
+        <v>44</v>
+      </c>
+      <c r="J80" s="22" t="inlineStr">
+        <is>
+          <t>SC/ST/BC/EWS 5 years; PwBD 10 years; ex-servicemen and regular AP Government employees as per A.P. State and Subordinate Service Rules (relaxation details in the Detailed Notification)</t>
+        </is>
+      </c>
+      <c r="K80" s="22" t="inlineStr">
+        <is>
+          <t>06/11/2026 to 26/11/2026 (11:59 PM)</t>
+        </is>
+      </c>
+      <c r="L80" s="22" t="inlineStr">
+        <is>
+          <t>2026-11-26</t>
+        </is>
+      </c>
+      <c r="M80" s="22" t="inlineStr">
+        <is>
+          <t>tba (single-level CBRT, no screening test)</t>
+        </is>
+      </c>
+      <c r="N80" s="22" t="inlineStr">
+        <is>
+          <t>https://psc.ap.gov.in</t>
+        </is>
+      </c>
+      <c r="O80" s="22" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="P80" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="Q80" s="22" t="inlineStr">
+        <is>
+          <t>Brief notification dated 13/10/2026; applications open 06/11/2026; detailed notification due on or before 06/11/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="B81" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh Public Service Commission (APPSC)</t>
+        </is>
+      </c>
+      <c r="C81" s="22" t="inlineStr">
+        <is>
+          <t>Notification No. 33/2026 - Royalty Inspector, A.P. Mines and Geology Service</t>
+        </is>
+      </c>
+      <c r="D81" s="22" t="inlineStr">
+        <is>
+          <t>recruitment</t>
+        </is>
+      </c>
+      <c r="E81" s="22" t="inlineStr">
+        <is>
+          <t>9 provisional vacancies - Royalty Inspector, pay Rs 45,830 - 1,30,580</t>
+        </is>
+      </c>
+      <c r="F81" s="22" t="inlineStr">
+        <is>
+          <t>Educational qualification will be given in the Detailed Notification, due on or before 06/11/2026</t>
+        </is>
+      </c>
+      <c r="G81" s="22" t="inlineStr">
+        <is>
+          <t>18-44 years (Age as on 01/07/2026)</t>
+        </is>
+      </c>
+      <c r="H81" s="22" t="n">
+        <v>18</v>
+      </c>
+      <c r="I81" s="22" t="n">
+        <v>44</v>
+      </c>
+      <c r="J81" s="22" t="inlineStr">
+        <is>
+          <t>SC/ST/BC/EWS 5 years; PwBD 10 years; ex-servicemen and regular AP Government employees as per A.P. State and Subordinate Service Rules (relaxation details in the Detailed Notification)</t>
+        </is>
+      </c>
+      <c r="K81" s="22" t="inlineStr">
+        <is>
+          <t>06/11/2026 to 26/11/2026 (11:59 PM)</t>
+        </is>
+      </c>
+      <c r="L81" s="22" t="inlineStr">
+        <is>
+          <t>2026-11-26</t>
+        </is>
+      </c>
+      <c r="M81" s="22" t="inlineStr">
+        <is>
+          <t>tba (single-level CBRT, no screening test)</t>
+        </is>
+      </c>
+      <c r="N81" s="22" t="inlineStr">
+        <is>
+          <t>https://psc.ap.gov.in</t>
+        </is>
+      </c>
+      <c r="O81" s="22" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="P81" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="Q81" s="22" t="inlineStr">
+        <is>
+          <t>Brief notification dated 13/10/2026; applications open 06/11/2026; qualification and community break-up to be published in the detailed notification</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="B82" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh Public Service Commission (APPSC)</t>
+        </is>
+      </c>
+      <c r="C82" s="22" t="inlineStr">
+        <is>
+          <t>Notification No. 34/2026 - Lab Assistant, A.P. Mining Subordinate Service</t>
+        </is>
+      </c>
+      <c r="D82" s="22" t="inlineStr">
+        <is>
+          <t>recruitment</t>
+        </is>
+      </c>
+      <c r="E82" s="22" t="inlineStr">
+        <is>
+          <t>1 provisional vacancy - Lab Assistant in A.P. Mining Subordinate Service, pay Rs 35,570 - 1,09,910</t>
+        </is>
+      </c>
+      <c r="F82" s="22" t="inlineStr">
+        <is>
+          <t>B.Sc degree with Chemistry from a university recognised by the UGC</t>
+        </is>
+      </c>
+      <c r="G82" s="22" t="inlineStr">
+        <is>
+          <t>The brief notification fixes only the age reckoning date (01/07/2026) and defers the age range to the Detailed Notification - left blank rather than guessed</t>
+        </is>
+      </c>
+      <c r="H82" s="22" t="inlineStr"/>
+      <c r="I82" s="22" t="inlineStr"/>
+      <c r="J82" s="22" t="inlineStr">
+        <is>
+          <t>SC/ST/BC/EWS 5 years; PwBD 10 years; ex-servicemen and regular AP Government employees as per A.P. State and Subordinate Service Rules (relaxation details in the Detailed Notification)</t>
+        </is>
+      </c>
+      <c r="K82" s="22" t="inlineStr">
+        <is>
+          <t>06/11/2026 to 26/11/2026 (11:59 PM)</t>
+        </is>
+      </c>
+      <c r="L82" s="22" t="inlineStr">
+        <is>
+          <t>2026-11-26</t>
+        </is>
+      </c>
+      <c r="M82" s="22" t="inlineStr">
+        <is>
+          <t>tba (single-level CBRT, no screening test)</t>
+        </is>
+      </c>
+      <c r="N82" s="22" t="inlineStr">
+        <is>
+          <t>https://psc.ap.gov.in</t>
+        </is>
+      </c>
+      <c r="O82" s="22" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="P82" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="Q82" s="22" t="inlineStr">
+        <is>
+          <t>Brief notification dated 13/10/2026; unlike the companion Mines notifications this one does not state the age range in the brief notice; detailed notification due on or before 06/11/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="B83" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh Public Service Commission (APPSC)</t>
+        </is>
+      </c>
+      <c r="C83" s="22" t="inlineStr">
+        <is>
+          <t>Notification No. 35/2026 - Assistant Chemical Examiner, A.P. Prohibition and Excise Subordinate Service</t>
+        </is>
+      </c>
+      <c r="D83" s="22" t="inlineStr">
+        <is>
+          <t>recruitment</t>
+        </is>
+      </c>
+      <c r="E83" s="22" t="inlineStr">
+        <is>
+          <t>9 provisional vacancies - Assistant Chemical Examiner, pay Rs 40,970 - 1,24,380</t>
+        </is>
+      </c>
+      <c r="F83" s="22" t="inlineStr">
+        <is>
+          <t>Bachelor's Degree in Science with Chemistry, or B.Sc (Pharmacy), from a recognised university or equivalent</t>
+        </is>
+      </c>
+      <c r="G83" s="22" t="inlineStr">
+        <is>
+          <t>18-44 years (Age as on 01/07/2026)</t>
+        </is>
+      </c>
+      <c r="H83" s="22" t="n">
+        <v>18</v>
+      </c>
+      <c r="I83" s="22" t="n">
+        <v>44</v>
+      </c>
+      <c r="J83" s="22" t="inlineStr">
+        <is>
+          <t>SC/ST/BC/EWS 5 years; PwBD 10 years; ex-servicemen and regular AP Government employees as per A.P. State and Subordinate Service Rules (relaxation details in the Detailed Notification)</t>
+        </is>
+      </c>
+      <c r="K83" s="22" t="inlineStr">
+        <is>
+          <t>06/11/2026 to 26/11/2026 (11:59 PM)</t>
+        </is>
+      </c>
+      <c r="L83" s="22" t="inlineStr">
+        <is>
+          <t>2026-11-26</t>
+        </is>
+      </c>
+      <c r="M83" s="22" t="inlineStr">
+        <is>
+          <t>tba (single-level CBRT, no screening test)</t>
+        </is>
+      </c>
+      <c r="N83" s="22" t="inlineStr">
+        <is>
+          <t>https://psc.ap.gov.in</t>
+        </is>
+      </c>
+      <c r="O83" s="22" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="P83" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="Q83" s="22" t="inlineStr">
+        <is>
+          <t>Brief notification dated 13/10/2026; applications open 06/11/2026; detailed notification due on or before 06/11/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="B84" s="22" t="inlineStr">
+        <is>
+          <t>Andhra Pradesh Public Service Commission (APPSC)</t>
+        </is>
+      </c>
+      <c r="C84" s="22" t="inlineStr">
+        <is>
+          <t>Notification No. 36/2026 - Assistant Motor Vehicle Inspector, A.P. Transport Service</t>
+        </is>
+      </c>
+      <c r="D84" s="22" t="inlineStr">
+        <is>
+          <t>recruitment</t>
+        </is>
+      </c>
+      <c r="E84" s="22" t="inlineStr">
+        <is>
+          <t>50 provisional vacancies - Assistant Motor Vehicle Inspector, pay Rs 48,440 - 1,37,220</t>
+        </is>
+      </c>
+      <c r="F84" s="22" t="inlineStr">
+        <is>
+          <t>Degree in Mechanical or Automobile Engineering, OR Diploma in Automobile Engineering from SBTET Andhra Pradesh / Technological Diploma Examination Board Hyderabad or equivalent; plus a motor driving licence with at least 3 years driving experience and a Heavy Transport Vehicle endorsement (2 years accepted where 3-year candidates are unavailable). Women holding only an LMV licence must acquire the HTV endorsement within two years of joining</t>
+        </is>
+      </c>
+      <c r="G84" s="22" t="inlineStr">
+        <is>
+          <t>21-36 years (Age as on 01/07/2026)</t>
+        </is>
+      </c>
+      <c r="H84" s="22" t="n">
+        <v>21</v>
+      </c>
+      <c r="I84" s="22" t="n">
+        <v>36</v>
+      </c>
+      <c r="J84" s="22" t="inlineStr">
+        <is>
+          <t>SC/ST/BC/EWS 5 years; PwBD 10 years; ex-servicemen and regular AP Government employees as per A.P. State and Subordinate Service Rules (relaxation details in the Detailed Notification)</t>
+        </is>
+      </c>
+      <c r="K84" s="22" t="inlineStr">
+        <is>
+          <t>06/11/2026 to 26/11/2026 (11:59 PM)</t>
+        </is>
+      </c>
+      <c r="L84" s="22" t="inlineStr">
+        <is>
+          <t>2026-11-26</t>
+        </is>
+      </c>
+      <c r="M84" s="22" t="inlineStr">
+        <is>
+          <t>tba (single-level CBRT, no screening test)</t>
+        </is>
+      </c>
+      <c r="N84" s="22" t="inlineStr">
+        <is>
+          <t>https://psc.ap.gov.in</t>
+        </is>
+      </c>
+      <c r="O84" s="22" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="P84" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="Q84" s="22" t="inlineStr">
+        <is>
+          <t>Brief notification dated 13/10/2026; applications open 06/11/2026; physical requirements and community break-up to be given in the detailed notification due on or before 06/11/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="22" t="inlineStr">
+        <is>
+          <t>Central Govt</t>
+        </is>
+      </c>
+      <c r="B85" s="22" t="inlineStr">
+        <is>
+          <t>NTA (for the Department of Higher Education, Ministry of Education)</t>
+        </is>
+      </c>
+      <c r="C85" s="22" t="inlineStr">
+        <is>
+          <t>Joint Entrance Examination (Main) - 2027, Session 1 (January 2027)</t>
+        </is>
+      </c>
+      <c r="D85" s="22" t="inlineStr">
+        <is>
+          <t>entrance-exam</t>
+        </is>
+      </c>
+      <c r="E85" s="22" t="inlineStr">
+        <is>
+          <t>Paper 1 (B.E./B.Tech) and Paper 2A (B.Arch) / 2B (B.Planning) - admission to NITs, IIITs and other centrally funded technical institutions, and the eligibility test for JEE (Advanced)</t>
+        </is>
+      </c>
+      <c r="F85" s="22" t="inlineStr">
+        <is>
+          <t>Pass in Class 12 (or equivalent) as per the JEE (Main) 2027 Information Bulletin - eligibility is fixed by the year of passing the qualifying examination</t>
+        </is>
+      </c>
+      <c r="G85" s="22" t="inlineStr">
+        <is>
+          <t>No age range is prescribed in the public notice - eligibility for JEE (Main) 2027 is determined by the year of passing the Class 12 qualifying examination, so no numeric age limit is shown</t>
+        </is>
+      </c>
+      <c r="H85" s="22" t="inlineStr"/>
+      <c r="I85" s="22" t="inlineStr"/>
+      <c r="J85" s="22" t="inlineStr">
+        <is>
+          <t>Not applicable - no age limit prescribed</t>
+        </is>
+      </c>
+      <c r="K85" s="22" t="inlineStr">
+        <is>
+          <t>24/10/2026 to 22/11/2026 (11:50 PM); late fee window 23/11/2026 to 26/11/2026; correction in particulars 27/11/2026 to 29/11/2026</t>
+        </is>
+      </c>
+      <c r="L85" s="22" t="inlineStr">
+        <is>
+          <t>2026-11-22</t>
+        </is>
+      </c>
+      <c r="M85" s="22" t="inlineStr">
+        <is>
+          <t>20, 21, 22, 23, 24 and 28 January 2027 (Session 1); city intimation slip 30/12/2026, admit cards from 13/01/2027</t>
+        </is>
+      </c>
+      <c r="N85" s="22" t="inlineStr">
+        <is>
+          <t>https://jeemain.nta.nic.in/</t>
+        </is>
+      </c>
+      <c r="O85" s="22" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="P85" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="Q85" s="22" t="inlineStr">
+        <is>
+          <t>Public notice dated 24/10/2026; Session 2 (April 2027) applications run 05/01/2027 to 03/02/2027 under a separate notice; the exam is held in 13 languages including Telugu; one application only per candidate</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="22" t="inlineStr">
+        <is>
+          <t>Central Govt</t>
+        </is>
+      </c>
+      <c r="B86" s="22" t="inlineStr">
+        <is>
+          <t>UPSC</t>
+        </is>
+      </c>
+      <c r="C86" s="22" t="inlineStr">
+        <is>
+          <t>Special Advertisement No. 51/2026 - Principal and Vice-Principal, Education Department, Government of NCT of Delhi</t>
+        </is>
+      </c>
+      <c r="D86" s="22" t="inlineStr">
+        <is>
+          <t>recruitment</t>
+        </is>
+      </c>
+      <c r="E86" s="22" t="inlineStr">
+        <is>
+          <t>828 posts (Principal 124 - UR 69, EWS 11, OBC 18, SC 16, ST 10; Vice-Principal 704 - UR 287, EWS 71, OBC 189, SC 103, ST 54)</t>
+        </is>
+      </c>
+      <c r="F86" s="22" t="inlineStr">
+        <is>
+          <t>Master's Degree and Bachelor of Education from a recognised university/institute. Principal: ten years' teaching experience as Vice-Principal/PGT/TGT in a recognised high/higher secondary school or college. Vice-Principal: two years as PGT or three years as TGT. Doctorate and administrative charge desirable</t>
+        </is>
+      </c>
+      <c r="G86" s="22" t="inlineStr">
+        <is>
+          <t>Principal: 50 years for UR/EWS, 53 years for OBC and 55 years for SC/ST. Vice-Principal: 35 years for UR/EWS, 38 years for OBC and 40 years for SC/ST. Relaxable up to 10 years for PwBD subject to a maximum of 56 years</t>
+        </is>
+      </c>
+      <c r="H86" s="22" t="inlineStr"/>
+      <c r="I86" s="22" t="n">
+        <v>55</v>
+      </c>
+      <c r="J86" s="22" t="inlineStr">
+        <is>
+          <t>SC/ST 5 years; OBC 3 years; PwBD up to 10 years (maximum age 56); OBC reservation only against a certificate issued by the Government of NCT of Delhi</t>
+        </is>
+      </c>
+      <c r="K86" s="22" t="inlineStr">
+        <is>
+          <t>25/07/2026 to 14/08/2026, extended to 17/08/2026 (18:00 hrs); crucial date for age and eligibility remained 14/08/2026</t>
+        </is>
+      </c>
+      <c r="L86" s="22" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="M86" s="22" t="inlineStr">
+        <is>
+          <t>Pen-and-paper Combined Recruitment Test (CRT) on 01/11/2026 for shortlisting, followed by interview</t>
+        </is>
+      </c>
+      <c r="N86" s="22" t="inlineStr">
+        <is>
+          <t>https://www.upsc.gov.in/sites/default/files/AdvtNo-51-2026-Special-Engl-240726.pdf</t>
+        </is>
+      </c>
+      <c r="O86" s="22" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="P86" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="Q86" s="22" t="inlineStr">
+        <is>
+          <t>Applications closed 17/08/2026; the shortlisting CRT is scheduled for 01/11/2026, so admit-card and exam-city notices are the live items to watch; max age shown is the Principal UR/EWS limit</t>
         </is>
       </c>
     </row>

</xml_diff>